<commit_message>
Formulario: declaracion de Gemini (API gratuita), app de Claude y Perplexity
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/methods_description_form.xlsx
+++ b/docs/methods_description_form.xlsx
@@ -723,7 +723,9 @@
         <is>
           <t>• Claude Code (Sonnet and Opus), Anthropic, Claude Pro plan, consumer terms, "Help improve Claude" disabled (K. García).
 • Claude Code, Anthropic, Claude Pro plan, consumer terms, "Help improve Claude" disabled (L. Vargas).
-• Gemini through LangChain (notebook 06), Google, [TO COMPLETE: plan and data setting; who used it]. Received only target names and public database results, no patient data; its draft was not used as the final list.
+• Gemini 3.5-flash-lite and 3.8-flash (API through LangChain, notebook 06), Google, free tier of the API: content sent and responses may be used by Google to improve its products and may be read by human reviewers. Used by the team for an early draft of drug ideas, not used as the final list. Received only the disease name, the gene BUB1B, therapeutic target names and public database results; no patient data.
+• Claude (app), Anthropic, free plan, [TO CONFIRM: "Help improve Claude" setting]. Literature search on the disease and its treatments; no patient data.
+• Perplexity, Perplexity AI, free plan, [TO CONFIRM: data retention setting]. Literature search on the disease and its treatments; no patient data.
 All AI-generated statements were verified against primary sources (PubMed, Drugs@FDA, gnomAD, UniProt).</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Formulario oficial: version de Laura en envios/track2; app de Claude y Perplexity sin verificar
El formulario de docs/ (sincronizado con el informe en ingles, 200 horas-persona)
queda como el oficial y se copia a envios/track2/. Ojo: scripts/llenar_formulario.py
escribe en esa misma ruta; no correrlo sin volver a copiar esta version.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/methods_description_form.xlsx
+++ b/docs/methods_description_form.xlsx
@@ -724,8 +724,8 @@
           <t>• Claude Code (Sonnet and Opus), Anthropic, Claude Pro plan, consumer terms, "Help improve Claude" disabled (K. García).
 • Claude Code, Anthropic, Claude Pro plan, consumer terms, "Help improve Claude" disabled (L. Vargas).
 • Gemini 3.5-flash-lite and 3.8-flash (API through LangChain, notebook 06), Google, free tier of the API: content sent and responses may be used by Google to improve its products and may be read by human reviewers. Used by the team for an early draft of drug ideas, not used as the final list. Received only the disease name, the gene BUB1B, therapeutic target names and public database results; no patient data.
-• Claude (app), Anthropic, free plan, [TO CONFIRM: "Help improve Claude" setting]. Literature search on the disease and its treatments; no patient data.
-• Perplexity, Perplexity AI, free plan, [TO CONFIRM: data retention setting]. Literature search on the disease and its treatments; no patient data.
+• Claude (app), Anthropic, free plan; "Help improve Claude" setting not verified. Literature search on the disease and its treatments; no patient data.
+• Perplexity, Perplexity AI, free plan; data retention setting not verified. Literature search on the disease and its treatments; no patient data.
 All AI-generated statements were verified against primary sources (PubMed, Drugs@FDA, gnomAD, UniProt).</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Formulario: solo la hoja Track 2 (el equipo no participa en Track 1)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/methods_description_form.xlsx
+++ b/docs/methods_description_form.xlsx
@@ -6,8 +6,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="27480" yWindow="15680" windowWidth="42340" windowHeight="26880" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 1 methods" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 2 methods" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track 2 methods" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -198,22 +197,6 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>MVA Hackathon Organizers</author>
-  </authors>
-  <commentList>
-    <comment ref="B7" authorId="0" shapeId="0">
-      <text>
-        <t>Yellow cells are for your answers.
-Example: "HelixSquad"</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -503,156 +486,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
-  <cols>
-    <col width="85.1640625" customWidth="1" style="7" min="1" max="1"/>
-    <col width="45" customWidth="1" style="7" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16" customHeight="1" s="7">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Methods description — MVA Hackathon 2026, Track 1 (Variant Prediction)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="70" customHeight="1" s="7">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Please submit your answers with your Track 1 submission. All questions (with the exception of Question 1, in red) are voluntary; however, submissions without a methods description may be judged less favorably on the Innovation and Scalability criteria, since the panel can't assess what it can't see.
-Fill out this form once per model/approach submitted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="6" ht="16" customHeight="1" s="7">
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>Answers</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Team name</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Model number (fill out this form once per model/approach submitted; up to 6)</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Please describe your model/approach in detail.</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n"/>
-    </row>
-    <row r="10" ht="45" customHeight="1" s="7">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>(required) If commercially-available Generative AI was used, record the provider, the plan or tier, and the relevant setting in your methods description. A line is enough, for example, "Anthropic API, Claude Sonnet, commercial terms, no training on customer content."</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n"/>
-    </row>
-    <row r="11" ht="30" customHeight="1" s="7">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Please state whether the submission file is the automated output of your computational approach (preferred), or if it has undergone downstream manual review and curation.</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Please describe any downstream manual review in detail.</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n"/>
-    </row>
-    <row r="13" ht="45" customHeight="1" s="7">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Please state whether your approach only used publicly available data (preferred) or if proprietary data was also used. If proprietary data were used, where possible, please also include a submission based only on publicly available data.</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n"/>
-    </row>
-    <row r="14" ht="30" customHeight="1" s="7">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Please describe any public data used in detail (e.g., reference panels, population databases, literature).</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Please describe any proprietary data used in detail.</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n"/>
-    </row>
-    <row r="16" ht="30" customHeight="1" s="7">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Is your approach able to output proposed pairs of compound heterozygous candidate variants, or only single candidate variants?</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n"/>
-    </row>
-    <row r="17" ht="30" customHeight="1" s="7">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>How did you handle secondary or incidental findings, if any? (See the finding_type column in your submission.)</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Please provide an estimate of run time and cost for your approach (if possible).</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="n"/>
-    </row>
-    <row r="19" ht="30" customHeight="1" s="7">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Provide a method abstract (up to 500 words). Please include strengths and limitations of your method as well as methodological detail.</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:B4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>

</xml_diff>